<commit_message>
Super Saiyan Engineer Jo 🔥
Major update, starting to come together rather nicely!
-Finally generates functional files

p.s. Need to add:
-transom functionality before tomorrow's FAT
-panel fab macros logic
</commit_message>
<xml_diff>
--- a/VPD PO download generator/trying stuff business systems.xlsx
+++ b/VPD PO download generator/trying stuff business systems.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jwa25\source\repos\VPD PO download generator\VPD PO download generator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F64DD68B-9A2A-416B-9829-5C44E5247874}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9750C3A5-C3C5-4EB7-9227-5D2875E77025}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{D51960FC-1269-4ACE-8C84-C0CBF6215B21}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{D51960FC-1269-4ACE-8C84-C0CBF6215B21}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1388" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1397" uniqueCount="148">
   <si>
     <t>KSO5088990 PVPDFJB    TWHWHNA01AA001CR-SO-5088990-1-1                                            L07975</t>
   </si>
@@ -447,6 +447,33 @@
   </si>
   <si>
     <t>7,7</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> profileID: str</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> length: float</t>
+  </si>
+  <si>
+    <t>Handing</t>
+  </si>
+  <si>
+    <t>frameWelderQRCode</t>
+  </si>
+  <si>
+    <t>panelWelderQRCode</t>
+  </si>
+  <si>
+    <t>cartID</t>
+  </si>
+  <si>
+    <t>cartBin</t>
+  </si>
+  <si>
+    <t>panelComponentsNeeded</t>
+  </si>
+  <si>
+    <t>panelComponentsCut</t>
   </si>
 </sst>
 </file>
@@ -740,7 +767,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -813,6 +840,13 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -8123,44 +8157,44 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D31D181-2758-43CB-B29A-A87F826596E0}">
-  <dimension ref="A3:Q52"/>
+  <dimension ref="A3:U52"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.140625" customWidth="1"/>
     <col min="2" max="2" width="28.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17.7109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="24.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="27.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="27.5703125" customWidth="1"/>
     <col min="6" max="6" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="24.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16" customWidth="1"/>
     <col min="9" max="9" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="23" customWidth="1"/>
-    <col min="14" max="14" width="1.5703125" customWidth="1"/>
-    <col min="15" max="15" width="18.140625" customWidth="1"/>
-    <col min="16" max="16" width="1.42578125" customWidth="1"/>
-    <col min="17" max="17" width="45.85546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="23" customWidth="1"/>
+    <col min="18" max="18" width="1.5703125" customWidth="1"/>
+    <col min="19" max="19" width="18.140625" customWidth="1"/>
+    <col min="20" max="20" width="1.42578125" customWidth="1"/>
+    <col min="21" max="21" width="45.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>104</v>
       </c>
-      <c r="M7" s="23" t="s">
-        <v>107</v>
-      </c>
-      <c r="O7" s="23" t="s">
-        <v>107</v>
-      </c>
       <c r="Q7" s="23" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="8" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="S7" s="23" t="s">
+        <v>107</v>
+      </c>
+      <c r="U7" s="23" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="8" spans="1:21" ht="63" x14ac:dyDescent="0.25">
       <c r="B8" s="20" t="s">
         <v>91</v>
       </c>
@@ -8185,17 +8219,38 @@
       <c r="I8" s="20" t="s">
         <v>97</v>
       </c>
-      <c r="M8" s="26" t="s">
+      <c r="J8" s="51" t="s">
+        <v>141</v>
+      </c>
+      <c r="K8" s="51" t="s">
+        <v>144</v>
+      </c>
+      <c r="L8" t="s">
+        <v>145</v>
+      </c>
+      <c r="M8" s="52" t="s">
+        <v>142</v>
+      </c>
+      <c r="N8" s="52" t="s">
+        <v>143</v>
+      </c>
+      <c r="O8" s="52" t="s">
+        <v>146</v>
+      </c>
+      <c r="P8" s="53" t="s">
+        <v>147</v>
+      </c>
+      <c r="Q8" s="26" t="s">
         <v>108</v>
       </c>
-      <c r="O8" s="26" t="s">
+      <c r="S8" s="26" t="s">
         <v>114</v>
       </c>
-      <c r="Q8" s="26" t="s">
+      <c r="U8" s="26" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>98</v>
       </c>
@@ -8220,17 +8275,17 @@
       <c r="I9" t="s">
         <v>102</v>
       </c>
-      <c r="M9" s="24" t="s">
+      <c r="Q9" s="24" t="s">
         <v>109</v>
       </c>
-      <c r="O9" s="24" t="s">
+      <c r="S9" s="24" t="s">
         <v>115</v>
       </c>
-      <c r="Q9" s="24" t="s">
+      <c r="U9" s="24" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>103</v>
       </c>
@@ -8255,38 +8310,44 @@
       <c r="I10" t="s">
         <v>102</v>
       </c>
-      <c r="M10" s="24" t="s">
+      <c r="Q10" s="24" t="s">
         <v>110</v>
       </c>
-      <c r="O10" s="25" t="s">
+      <c r="S10" s="25" t="s">
         <v>116</v>
       </c>
-      <c r="Q10" s="24" t="s">
+      <c r="U10" s="24" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="M11" s="24" t="s">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="Q11" s="24" t="s">
         <v>111</v>
       </c>
-      <c r="Q11" s="24" t="s">
+      <c r="U11" s="24" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="M12" s="24" t="s">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="Q12" s="24" t="s">
         <v>112</v>
       </c>
-      <c r="Q12" s="25" t="s">
+      <c r="S12" t="s">
+        <v>139</v>
+      </c>
+      <c r="U12" s="25" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="M13" s="25" t="s">
+    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="Q13" s="25" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="S13" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>105</v>
       </c>

</xml_diff>